<commit_message>
`Refactor API and OCR logic: update dependencies, remove unused code, and modify file structure`
</commit_message>
<xml_diff>
--- a/wardpdf/API/output/voter_data_4-54.xlsx
+++ b/wardpdf/API/output/voter_data_4-54.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,20 +456,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>SexAge</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Age</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Page</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>RectIndex</t>
         </is>
@@ -501,14 +496,17 @@
           <t>ഈറപ്പാക്കല്‍</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
-      <c r="I2" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -536,12 +534,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
       <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -571,12 +572,15 @@
           <t>കെ ആര്‍ നാരായണന്‍ ചെങ്ങറ</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ളി</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
       <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -606,12 +610,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ay75</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
       <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
         <v>5</v>
       </c>
     </row>
@@ -643,14 +650,13 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>പൂ/72</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
       <c r="H6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -681,11 +687,10 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
       <c r="H7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" t="n">
         <v>7</v>
       </c>
     </row>
@@ -715,12 +720,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ay71</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
       <c r="H8" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" t="n">
         <v>8</v>
       </c>
     </row>
@@ -750,12 +758,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
       <c r="H9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" t="n">
         <v>9</v>
       </c>
     </row>
@@ -785,12 +796,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ay71</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
       <c r="H10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" t="n">
         <v>10</v>
       </c>
     </row>
@@ -820,12 +834,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ayv70</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
       <c r="H11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I11" t="n">
         <v>11</v>
       </c>
     </row>
@@ -857,14 +874,13 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>പൂ/70</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
       <c r="H12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I12" t="n">
         <v>12</v>
       </c>
     </row>
@@ -896,14 +912,13 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>പു/70</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
       <c r="H13" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" t="n">
         <v>13</v>
       </c>
     </row>
@@ -933,12 +948,15 @@
           <t>കെ ആര്‍ നാരായണന്‍ ചെങ്ങറ</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ക്നോള്ചനി</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
       <c r="H14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I14" t="n">
         <v>14</v>
       </c>
     </row>
@@ -968,12 +986,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/69</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
       <c r="H15" t="n">
-        <v>2</v>
-      </c>
-      <c r="I15" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1003,12 +1024,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/69</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
       <c r="H16" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1040,14 +1064,13 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>പു/68</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
       <c r="H17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1078,11 +1101,10 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
       <c r="H18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I18" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1112,12 +1134,15 @@
           <t>ചെങ്ങറ കലിയടുക്കം</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/68</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
       <c r="H19" t="n">
-        <v>2</v>
-      </c>
-      <c r="I19" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1147,12 +1172,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/67/</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
       <c r="H20" t="n">
-        <v>3</v>
-      </c>
-      <c r="I20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1182,12 +1210,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/67/</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>3</v>
+      </c>
       <c r="H21" t="n">
-        <v>3</v>
-      </c>
-      <c r="I21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1218,11 +1249,10 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
       <c r="H22" t="n">
-        <v>3</v>
-      </c>
-      <c r="I22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1252,14 +1282,17 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ay/65</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
       <c r="H23" t="n">
         <v>3</v>
       </c>
-      <c r="I23" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1287,12 +1320,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ay/64</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>3</v>
+      </c>
       <c r="H24" t="n">
-        <v>3</v>
-      </c>
-      <c r="I24" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1322,12 +1358,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ayvo4</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>3</v>
+      </c>
       <c r="H25" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1357,12 +1396,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/63</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>3</v>
+      </c>
       <c r="H26" t="n">
-        <v>3</v>
-      </c>
-      <c r="I26" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1392,12 +1434,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>3</v>
+      </c>
       <c r="H27" t="n">
-        <v>3</v>
-      </c>
-      <c r="I27" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1428,11 +1473,10 @@
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
       <c r="H28" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1462,12 +1506,15 @@
           <t>ചെങ്ങറ കലിയടുക്കം</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ay62</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
       <c r="H29" t="n">
-        <v>3</v>
-      </c>
-      <c r="I29" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1498,11 +1545,10 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>3</v>
+      </c>
       <c r="H30" t="n">
-        <v>3</v>
-      </c>
-      <c r="I30" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1532,12 +1578,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ay62</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
       <c r="H31" t="n">
-        <v>3</v>
-      </c>
-      <c r="I31" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1567,12 +1616,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ay61</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
       <c r="H32" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1603,11 +1655,10 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>3</v>
+      </c>
       <c r="H33" t="n">
-        <v>3</v>
-      </c>
-      <c r="I33" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1637,12 +1688,15 @@
           <t>4/54</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>റ്റി. കോളനി</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>3</v>
+      </c>
       <c r="H34" t="n">
-        <v>3</v>
-      </c>
-      <c r="I34" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1674,14 +1728,13 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
+          <t>പു/€0</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>3</v>
+      </c>
       <c r="H35" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1711,12 +1764,15 @@
           <t>ചെങ്ങറ കാലിയാടുക്കാം</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/60</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>3</v>
+      </c>
       <c r="H36" t="n">
-        <v>3</v>
-      </c>
-      <c r="I36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1746,12 +1802,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
       <c r="H37" t="n">
-        <v>3</v>
-      </c>
-      <c r="I37" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1781,12 +1840,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ay/57</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>3</v>
+      </c>
       <c r="H38" t="n">
-        <v>3</v>
-      </c>
-      <c r="I38" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1816,12 +1878,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>3</v>
+      </c>
       <c r="H39" t="n">
-        <v>3</v>
-      </c>
-      <c r="I39" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1851,12 +1916,15 @@
           <t>ഈരപ്പാക്കല്‍ വീട്‌</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
       <c r="H40" t="n">
-        <v>4</v>
-      </c>
-      <c r="I40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1888,14 +1956,13 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>പു/4</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>4</v>
+      </c>
       <c r="H41" t="n">
-        <v>4</v>
-      </c>
-      <c r="I41" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1925,12 +1992,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
       <c r="H42" t="n">
-        <v>4</v>
-      </c>
-      <c r="I42" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1961,11 +2031,10 @@
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>4</v>
+      </c>
       <c r="H43" t="n">
-        <v>4</v>
-      </c>
-      <c r="I43" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1995,14 +2064,17 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/2</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>4</v>
+      </c>
       <c r="H44" t="n">
         <v>4</v>
       </c>
-      <c r="I44" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2032,14 +2104,13 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ൂ</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>ഹദൂ്സിംങ്ങ്‌ കോളനി</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>4</v>
+      </c>
       <c r="H45" t="n">
-        <v>4</v>
-      </c>
-      <c r="I45" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2069,12 +2140,15 @@
           <t>ചെങ്ങറ</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>©</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>4</v>
+      </c>
       <c r="H46" t="n">
-        <v>4</v>
-      </c>
-      <c r="I46" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2104,12 +2178,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>oV/4l</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>4</v>
+      </c>
       <c r="H47" t="n">
-        <v>4</v>
-      </c>
-      <c r="I47" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2139,12 +2216,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>4</v>
+      </c>
       <c r="H48" t="n">
-        <v>4</v>
-      </c>
-      <c r="I48" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2174,12 +2254,15 @@
           <t>പുതുശേരിയില്‍</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>ayv/40</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>4</v>
+      </c>
       <c r="H49" t="n">
-        <v>4</v>
-      </c>
-      <c r="I49" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2209,12 +2292,15 @@
           <t>മാങ്കോട്ട്‌ കിഴക്കേതില്‍</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>വ</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>4</v>
+      </c>
       <c r="H50" t="n">
-        <v>4</v>
-      </c>
-      <c r="I50" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2244,12 +2330,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>ay 37</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>4</v>
+      </c>
       <c r="H51" t="n">
-        <v>4</v>
-      </c>
-      <c r="I51" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2279,12 +2368,15 @@
           <t>മാങ്കോട്ട്‌ കിഴക്കേതില്‍</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ay/37</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>4</v>
+      </c>
       <c r="H52" t="n">
-        <v>4</v>
-      </c>
-      <c r="I52" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2316,14 +2408,13 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>പ</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
+          <t>പു/37</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>4</v>
+      </c>
       <c r="H53" t="n">
-        <v>4</v>
-      </c>
-      <c r="I53" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2353,12 +2444,15 @@
           <t>ചെങ്ങറ കോളനി</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>വ്‌</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>4</v>
+      </c>
       <c r="H54" t="n">
-        <v>4</v>
-      </c>
-      <c r="I54" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2389,11 +2483,10 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="n">
+        <v>4</v>
+      </c>
       <c r="H55" t="n">
-        <v>4</v>
-      </c>
-      <c r="I55" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2423,12 +2516,15 @@
           <t>ചെറുകുന്നത്ത്‌, ചെങ്ങറ</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>സ്ത്രീ/27</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>4</v>
+      </c>
       <c r="H56" t="n">
-        <v>4</v>
-      </c>
-      <c r="I56" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2458,12 +2554,15 @@
           <t>ചെങ്ങറ</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ay23</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>4</v>
+      </c>
       <c r="H57" t="n">
-        <v>4</v>
-      </c>
-      <c r="I57" t="n">
         <v>17</v>
       </c>
     </row>

</xml_diff>